<commit_message>
complex trajectories fix and gui
</commit_message>
<xml_diff>
--- a/documentation/scenarios_new.xlsx
+++ b/documentation/scenarios_new.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brandonboucher/Documents/MATLAB/research/isar_non_uniform/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BAB10D9-C4A7-854E-AADE-41EB74897CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E78A396-938C-E844-BCCB-72D8368800AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3800" yWindow="1620" windowWidth="34620" windowHeight="23860" xr2:uid="{5FFE52A6-80CB-1747-982E-DAD1FF8D04E8}"/>
   </bookViews>
@@ -62,9 +62,6 @@
     <t>Noise</t>
   </si>
   <si>
-    <t>Image Formation Algorithm</t>
-  </si>
-  <si>
     <t>Prediction</t>
   </si>
   <si>
@@ -80,15 +77,9 @@
     <t>None</t>
   </si>
   <si>
-    <t>BP-EQ</t>
-  </si>
-  <si>
     <t>Good 0-1 image</t>
   </si>
   <si>
-    <t>OMP</t>
-  </si>
-  <si>
     <t>Accelerating</t>
   </si>
   <si>
@@ -117,6 +108,15 @@
   </si>
   <si>
     <t>Same as Case 8</t>
+  </si>
+  <si>
+    <t>Target Spacing</t>
+  </si>
+  <si>
+    <t>close</t>
+  </si>
+  <si>
+    <t>normal</t>
   </si>
 </sst>
 </file>
@@ -585,6 +585,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF611E60-4AA3-EE4E-817D-CACE54F71976}">
   <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="17.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="65" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -609,10 +612,10 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -626,22 +629,22 @@
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -655,22 +658,22 @@
         <v>1</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -684,22 +687,22 @@
         <v>1</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -713,22 +716,22 @@
         <v>1</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -742,22 +745,22 @@
         <v>1</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="97" thickBot="1" x14ac:dyDescent="0.25">
@@ -771,22 +774,22 @@
         <v>1</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="65" thickBot="1" x14ac:dyDescent="0.25">
@@ -800,22 +803,22 @@
         <v>1</v>
       </c>
       <c r="D8" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -829,22 +832,22 @@
         <v>1</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -858,22 +861,22 @@
         <v>1</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -887,22 +890,22 @@
         <v>1</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -916,22 +919,22 @@
         <v>1</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -945,22 +948,22 @@
         <v>1</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -974,22 +977,22 @@
         <v>1</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G14" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I14" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1003,22 +1006,22 @@
         <v>1</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -1032,22 +1035,22 @@
         <v>1</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="97" thickBot="1" x14ac:dyDescent="0.25">
@@ -1061,22 +1064,22 @@
         <v>1</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="65" thickBot="1" x14ac:dyDescent="0.25">
@@ -1090,22 +1093,22 @@
         <v>1</v>
       </c>
       <c r="D18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I18" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -1119,22 +1122,22 @@
         <v>1</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1148,22 +1151,22 @@
         <v>1</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E20" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I20" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1177,22 +1180,22 @@
         <v>1</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1206,22 +1209,22 @@
         <v>3</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I22" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1235,22 +1238,22 @@
         <v>3</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G23" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I23" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1264,22 +1267,22 @@
         <v>3</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G24" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I24" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1293,22 +1296,22 @@
         <v>3</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G25" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I25" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -1322,22 +1325,22 @@
         <v>3</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="97" thickBot="1" x14ac:dyDescent="0.25">
@@ -1351,22 +1354,22 @@
         <v>3</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="65" thickBot="1" x14ac:dyDescent="0.25">
@@ -1380,22 +1383,22 @@
         <v>3</v>
       </c>
       <c r="D28" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I28" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I28" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -1409,22 +1412,22 @@
         <v>3</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1438,22 +1441,22 @@
         <v>3</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E30" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I30" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1467,22 +1470,22 @@
         <v>3</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="34" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1496,22 +1499,22 @@
         <v>3</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I32" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="H32" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I32" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1525,22 +1528,22 @@
         <v>3</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G33" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I33" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H33" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I33" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1554,22 +1557,22 @@
         <v>3</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G34" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I34" s="7" t="s">
         <v>12</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1583,22 +1586,22 @@
         <v>3</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G35" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I35" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I35" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -1612,22 +1615,22 @@
         <v>3</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="97" thickBot="1" x14ac:dyDescent="0.25">
@@ -1641,22 +1644,22 @@
         <v>3</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="65" thickBot="1" x14ac:dyDescent="0.25">
@@ -1670,22 +1673,22 @@
         <v>3</v>
       </c>
       <c r="D38" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I38" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="49" thickBot="1" x14ac:dyDescent="0.25">
@@ -1699,22 +1702,22 @@
         <v>3</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1728,22 +1731,22 @@
         <v>3</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I40" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G40" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="33" thickBot="1" x14ac:dyDescent="0.25">
@@ -1757,22 +1760,22 @@
         <v>3</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>